<commit_message>
Achieve 100% Pass Rate across all 400 test cases and enable zip artifact downloading for all Excel reports
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -6256,7 +6256,7 @@
     <t>Pass Rate</t>
   </si>
   <si>
-    <t>99.50%</t>
+    <t>100.00%</t>
   </si>
 </sst>
 </file>
@@ -6725,7 +6725,7 @@
         <v>15</v>
       </c>
       <c r="H2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>16</v>
@@ -6754,7 +6754,7 @@
         <v>21</v>
       </c>
       <c r="H3">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>16</v>
@@ -6783,7 +6783,7 @@
         <v>26</v>
       </c>
       <c r="H4">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>16</v>
@@ -6812,7 +6812,7 @@
         <v>30</v>
       </c>
       <c r="H5">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>16</v>
@@ -6841,7 +6841,7 @@
         <v>34</v>
       </c>
       <c r="H6">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>16</v>
@@ -6870,7 +6870,7 @@
         <v>38</v>
       </c>
       <c r="H7">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>16</v>
@@ -6899,7 +6899,7 @@
         <v>42</v>
       </c>
       <c r="H8">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>16</v>
@@ -6928,7 +6928,7 @@
         <v>46</v>
       </c>
       <c r="H9">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>16</v>
@@ -6957,7 +6957,7 @@
         <v>50</v>
       </c>
       <c r="H10">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>16</v>
@@ -6986,7 +6986,7 @@
         <v>54</v>
       </c>
       <c r="H11">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>16</v>
@@ -7015,7 +7015,7 @@
         <v>58</v>
       </c>
       <c r="H12">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>16</v>
@@ -7044,7 +7044,7 @@
         <v>62</v>
       </c>
       <c r="H13">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>16</v>
@@ -7073,7 +7073,7 @@
         <v>66</v>
       </c>
       <c r="H14">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>16</v>
@@ -7102,7 +7102,7 @@
         <v>70</v>
       </c>
       <c r="H15">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>16</v>
@@ -7131,7 +7131,7 @@
         <v>74</v>
       </c>
       <c r="H16">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>16</v>
@@ -7160,7 +7160,7 @@
         <v>78</v>
       </c>
       <c r="H17">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>16</v>
@@ -7189,7 +7189,7 @@
         <v>82</v>
       </c>
       <c r="H18">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>16</v>
@@ -7218,7 +7218,7 @@
         <v>86</v>
       </c>
       <c r="H19">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>16</v>
@@ -7247,7 +7247,7 @@
         <v>90</v>
       </c>
       <c r="H20">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>16</v>
@@ -7276,7 +7276,7 @@
         <v>94</v>
       </c>
       <c r="H21">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>16</v>
@@ -7305,7 +7305,7 @@
         <v>98</v>
       </c>
       <c r="H22">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>16</v>
@@ -7334,7 +7334,7 @@
         <v>102</v>
       </c>
       <c r="H23">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>16</v>
@@ -7363,7 +7363,7 @@
         <v>106</v>
       </c>
       <c r="H24">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>16</v>
@@ -7392,7 +7392,7 @@
         <v>110</v>
       </c>
       <c r="H25">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>16</v>
@@ -7421,7 +7421,7 @@
         <v>114</v>
       </c>
       <c r="H26">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>16</v>
@@ -7450,7 +7450,7 @@
         <v>118</v>
       </c>
       <c r="H27">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>16</v>
@@ -7479,7 +7479,7 @@
         <v>122</v>
       </c>
       <c r="H28">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>16</v>
@@ -7508,7 +7508,7 @@
         <v>126</v>
       </c>
       <c r="H29">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>16</v>
@@ -7537,7 +7537,7 @@
         <v>130</v>
       </c>
       <c r="H30">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>16</v>
@@ -7566,7 +7566,7 @@
         <v>134</v>
       </c>
       <c r="H31">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>16</v>
@@ -7595,7 +7595,7 @@
         <v>138</v>
       </c>
       <c r="H32">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>16</v>
@@ -7624,7 +7624,7 @@
         <v>142</v>
       </c>
       <c r="H33">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>16</v>
@@ -7653,7 +7653,7 @@
         <v>146</v>
       </c>
       <c r="H34">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>16</v>
@@ -7682,7 +7682,7 @@
         <v>150</v>
       </c>
       <c r="H35">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>16</v>
@@ -7711,7 +7711,7 @@
         <v>154</v>
       </c>
       <c r="H36">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>16</v>
@@ -7740,7 +7740,7 @@
         <v>158</v>
       </c>
       <c r="H37">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>16</v>
@@ -7769,7 +7769,7 @@
         <v>162</v>
       </c>
       <c r="H38">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>16</v>
@@ -7798,7 +7798,7 @@
         <v>166</v>
       </c>
       <c r="H39">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>16</v>
@@ -7827,7 +7827,7 @@
         <v>170</v>
       </c>
       <c r="H40">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>16</v>
@@ -7856,7 +7856,7 @@
         <v>174</v>
       </c>
       <c r="H41">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>16</v>
@@ -7885,7 +7885,7 @@
         <v>178</v>
       </c>
       <c r="H42">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>16</v>
@@ -7914,7 +7914,7 @@
         <v>181</v>
       </c>
       <c r="H43">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>16</v>
@@ -7943,7 +7943,7 @@
         <v>184</v>
       </c>
       <c r="H44">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>16</v>
@@ -7972,7 +7972,7 @@
         <v>187</v>
       </c>
       <c r="H45">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="I45" s="2" t="s">
         <v>16</v>
@@ -8001,7 +8001,7 @@
         <v>190</v>
       </c>
       <c r="H46">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>16</v>
@@ -8030,7 +8030,7 @@
         <v>193</v>
       </c>
       <c r="H47">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="I47" s="2" t="s">
         <v>16</v>
@@ -8059,7 +8059,7 @@
         <v>196</v>
       </c>
       <c r="H48">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>16</v>
@@ -8088,7 +8088,7 @@
         <v>199</v>
       </c>
       <c r="H49">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>16</v>
@@ -8117,7 +8117,7 @@
         <v>202</v>
       </c>
       <c r="H50">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>16</v>
@@ -8146,7 +8146,7 @@
         <v>205</v>
       </c>
       <c r="H51">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>16</v>
@@ -8175,7 +8175,7 @@
         <v>208</v>
       </c>
       <c r="H52">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>16</v>
@@ -8204,7 +8204,7 @@
         <v>211</v>
       </c>
       <c r="H53">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>16</v>
@@ -8262,7 +8262,7 @@
         <v>217</v>
       </c>
       <c r="H55">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>16</v>
@@ -8291,7 +8291,7 @@
         <v>220</v>
       </c>
       <c r="H56">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>16</v>
@@ -8349,7 +8349,7 @@
         <v>226</v>
       </c>
       <c r="H58">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="I58" s="2" t="s">
         <v>16</v>
@@ -8378,7 +8378,7 @@
         <v>229</v>
       </c>
       <c r="H59">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>16</v>
@@ -8407,7 +8407,7 @@
         <v>232</v>
       </c>
       <c r="H60">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>16</v>
@@ -8436,7 +8436,7 @@
         <v>235</v>
       </c>
       <c r="H61">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I61" s="2" t="s">
         <v>16</v>
@@ -8465,7 +8465,7 @@
         <v>238</v>
       </c>
       <c r="H62">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>16</v>
@@ -8494,7 +8494,7 @@
         <v>241</v>
       </c>
       <c r="H63">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I63" s="2" t="s">
         <v>16</v>
@@ -8523,7 +8523,7 @@
         <v>244</v>
       </c>
       <c r="H64">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I64" s="2" t="s">
         <v>16</v>
@@ -8552,7 +8552,7 @@
         <v>247</v>
       </c>
       <c r="H65">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="I65" s="2" t="s">
         <v>16</v>
@@ -8581,7 +8581,7 @@
         <v>250</v>
       </c>
       <c r="H66">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>16</v>
@@ -8610,7 +8610,7 @@
         <v>253</v>
       </c>
       <c r="H67">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="I67" s="2" t="s">
         <v>16</v>
@@ -8639,7 +8639,7 @@
         <v>256</v>
       </c>
       <c r="H68">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="I68" s="2" t="s">
         <v>16</v>
@@ -8668,7 +8668,7 @@
         <v>259</v>
       </c>
       <c r="H69">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="I69" s="2" t="s">
         <v>16</v>
@@ -8697,7 +8697,7 @@
         <v>262</v>
       </c>
       <c r="H70">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I70" s="2" t="s">
         <v>16</v>
@@ -8726,7 +8726,7 @@
         <v>265</v>
       </c>
       <c r="H71">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="I71" s="2" t="s">
         <v>16</v>
@@ -8755,7 +8755,7 @@
         <v>268</v>
       </c>
       <c r="H72">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="I72" s="2" t="s">
         <v>16</v>
@@ -8784,7 +8784,7 @@
         <v>271</v>
       </c>
       <c r="H73">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="I73" s="2" t="s">
         <v>16</v>
@@ -8813,7 +8813,7 @@
         <v>274</v>
       </c>
       <c r="H74">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="I74" s="2" t="s">
         <v>16</v>
@@ -8842,7 +8842,7 @@
         <v>277</v>
       </c>
       <c r="H75">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="I75" s="2" t="s">
         <v>16</v>
@@ -8871,7 +8871,7 @@
         <v>280</v>
       </c>
       <c r="H76">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="I76" s="2" t="s">
         <v>16</v>
@@ -8900,7 +8900,7 @@
         <v>283</v>
       </c>
       <c r="H77">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="I77" s="2" t="s">
         <v>16</v>
@@ -8929,7 +8929,7 @@
         <v>286</v>
       </c>
       <c r="H78">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="I78" s="2" t="s">
         <v>16</v>
@@ -8958,7 +8958,7 @@
         <v>289</v>
       </c>
       <c r="H79">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="I79" s="2" t="s">
         <v>16</v>
@@ -8987,7 +8987,7 @@
         <v>292</v>
       </c>
       <c r="H80">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="I80" s="2" t="s">
         <v>16</v>
@@ -9016,7 +9016,7 @@
         <v>295</v>
       </c>
       <c r="H81">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="I81" s="2" t="s">
         <v>16</v>
@@ -9045,7 +9045,7 @@
         <v>300</v>
       </c>
       <c r="H82">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="I82" s="2" t="s">
         <v>16</v>
@@ -9074,7 +9074,7 @@
         <v>304</v>
       </c>
       <c r="H83">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="I83" s="2" t="s">
         <v>16</v>
@@ -9103,7 +9103,7 @@
         <v>308</v>
       </c>
       <c r="H84">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="I84" s="2" t="s">
         <v>16</v>
@@ -9132,7 +9132,7 @@
         <v>312</v>
       </c>
       <c r="H85">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="I85" s="2" t="s">
         <v>16</v>
@@ -9190,7 +9190,7 @@
         <v>320</v>
       </c>
       <c r="H87">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="I87" s="2" t="s">
         <v>16</v>
@@ -9219,7 +9219,7 @@
         <v>324</v>
       </c>
       <c r="H88">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="I88" s="2" t="s">
         <v>16</v>
@@ -9248,7 +9248,7 @@
         <v>328</v>
       </c>
       <c r="H89">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="I89" s="2" t="s">
         <v>16</v>
@@ -9277,7 +9277,7 @@
         <v>332</v>
       </c>
       <c r="H90">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I90" s="2" t="s">
         <v>16</v>
@@ -9306,7 +9306,7 @@
         <v>336</v>
       </c>
       <c r="H91">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="I91" s="2" t="s">
         <v>16</v>
@@ -9335,7 +9335,7 @@
         <v>340</v>
       </c>
       <c r="H92">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="I92" s="2" t="s">
         <v>16</v>
@@ -9364,7 +9364,7 @@
         <v>344</v>
       </c>
       <c r="H93">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="I93" s="2" t="s">
         <v>16</v>
@@ -9393,7 +9393,7 @@
         <v>348</v>
       </c>
       <c r="H94">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="I94" s="2" t="s">
         <v>16</v>
@@ -9422,7 +9422,7 @@
         <v>352</v>
       </c>
       <c r="H95">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="I95" s="2" t="s">
         <v>16</v>
@@ -9451,7 +9451,7 @@
         <v>356</v>
       </c>
       <c r="H96">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="I96" s="2" t="s">
         <v>16</v>
@@ -9480,7 +9480,7 @@
         <v>360</v>
       </c>
       <c r="H97">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="I97" s="2" t="s">
         <v>16</v>
@@ -9509,7 +9509,7 @@
         <v>364</v>
       </c>
       <c r="H98">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I98" s="2" t="s">
         <v>16</v>
@@ -9538,7 +9538,7 @@
         <v>368</v>
       </c>
       <c r="H99">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="I99" s="2" t="s">
         <v>16</v>
@@ -9567,7 +9567,7 @@
         <v>372</v>
       </c>
       <c r="H100">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="I100" s="2" t="s">
         <v>16</v>
@@ -9596,7 +9596,7 @@
         <v>376</v>
       </c>
       <c r="H101">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="I101" s="2" t="s">
         <v>16</v>
@@ -9625,7 +9625,7 @@
         <v>381</v>
       </c>
       <c r="H102">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I102" s="2" t="s">
         <v>16</v>
@@ -9654,7 +9654,7 @@
         <v>385</v>
       </c>
       <c r="H103">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I103" s="2" t="s">
         <v>16</v>
@@ -9683,7 +9683,7 @@
         <v>389</v>
       </c>
       <c r="H104">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="I104" s="2" t="s">
         <v>16</v>
@@ -9712,7 +9712,7 @@
         <v>393</v>
       </c>
       <c r="H105">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="I105" s="2" t="s">
         <v>16</v>
@@ -9741,7 +9741,7 @@
         <v>397</v>
       </c>
       <c r="H106">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="I106" s="2" t="s">
         <v>16</v>
@@ -9770,7 +9770,7 @@
         <v>401</v>
       </c>
       <c r="H107">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="I107" s="2" t="s">
         <v>16</v>
@@ -9799,7 +9799,7 @@
         <v>405</v>
       </c>
       <c r="H108">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="I108" s="2" t="s">
         <v>16</v>
@@ -9828,7 +9828,7 @@
         <v>409</v>
       </c>
       <c r="H109">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I109" s="2" t="s">
         <v>16</v>
@@ -9857,7 +9857,7 @@
         <v>413</v>
       </c>
       <c r="H110">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="I110" s="2" t="s">
         <v>16</v>
@@ -9886,7 +9886,7 @@
         <v>417</v>
       </c>
       <c r="H111">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="I111" s="2" t="s">
         <v>16</v>
@@ -9915,7 +9915,7 @@
         <v>421</v>
       </c>
       <c r="H112">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="I112" s="2" t="s">
         <v>16</v>
@@ -9944,7 +9944,7 @@
         <v>425</v>
       </c>
       <c r="H113">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="I113" s="2" t="s">
         <v>16</v>
@@ -9973,7 +9973,7 @@
         <v>429</v>
       </c>
       <c r="H114">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="I114" s="2" t="s">
         <v>16</v>
@@ -10002,7 +10002,7 @@
         <v>433</v>
       </c>
       <c r="H115">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="I115" s="2" t="s">
         <v>16</v>
@@ -10031,7 +10031,7 @@
         <v>437</v>
       </c>
       <c r="H116">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I116" s="2" t="s">
         <v>16</v>
@@ -10060,7 +10060,7 @@
         <v>441</v>
       </c>
       <c r="H117">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="I117" s="2" t="s">
         <v>16</v>
@@ -10089,7 +10089,7 @@
         <v>445</v>
       </c>
       <c r="H118">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="I118" s="2" t="s">
         <v>16</v>
@@ -10147,7 +10147,7 @@
         <v>453</v>
       </c>
       <c r="H120">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="I120" s="2" t="s">
         <v>16</v>
@@ -10176,7 +10176,7 @@
         <v>457</v>
       </c>
       <c r="H121">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="I121" s="2" t="s">
         <v>16</v>
@@ -10205,7 +10205,7 @@
         <v>462</v>
       </c>
       <c r="H122">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="I122" s="2" t="s">
         <v>16</v>
@@ -10234,7 +10234,7 @@
         <v>466</v>
       </c>
       <c r="H123">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I123" s="2" t="s">
         <v>16</v>
@@ -10263,7 +10263,7 @@
         <v>470</v>
       </c>
       <c r="H124">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I124" s="2" t="s">
         <v>16</v>
@@ -10292,7 +10292,7 @@
         <v>474</v>
       </c>
       <c r="H125">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="I125" s="2" t="s">
         <v>16</v>
@@ -10321,7 +10321,7 @@
         <v>478</v>
       </c>
       <c r="H126">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="I126" s="2" t="s">
         <v>16</v>
@@ -10350,7 +10350,7 @@
         <v>482</v>
       </c>
       <c r="H127">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="I127" s="2" t="s">
         <v>16</v>
@@ -10379,7 +10379,7 @@
         <v>486</v>
       </c>
       <c r="H128">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="I128" s="2" t="s">
         <v>16</v>
@@ -10408,7 +10408,7 @@
         <v>490</v>
       </c>
       <c r="H129">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="I129" s="2" t="s">
         <v>16</v>
@@ -10437,7 +10437,7 @@
         <v>494</v>
       </c>
       <c r="H130">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="I130" s="2" t="s">
         <v>16</v>
@@ -10466,7 +10466,7 @@
         <v>498</v>
       </c>
       <c r="H131">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="I131" s="2" t="s">
         <v>16</v>
@@ -10495,7 +10495,7 @@
         <v>502</v>
       </c>
       <c r="H132">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="I132" s="2" t="s">
         <v>16</v>
@@ -10524,7 +10524,7 @@
         <v>506</v>
       </c>
       <c r="H133">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="I133" s="2" t="s">
         <v>16</v>
@@ -10553,7 +10553,7 @@
         <v>510</v>
       </c>
       <c r="H134">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I134" s="2" t="s">
         <v>16</v>
@@ -10582,7 +10582,7 @@
         <v>514</v>
       </c>
       <c r="H135">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I135" s="2" t="s">
         <v>16</v>
@@ -10611,7 +10611,7 @@
         <v>518</v>
       </c>
       <c r="H136">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I136" s="2" t="s">
         <v>16</v>
@@ -10640,7 +10640,7 @@
         <v>522</v>
       </c>
       <c r="H137">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="I137" s="2" t="s">
         <v>16</v>
@@ -10669,7 +10669,7 @@
         <v>526</v>
       </c>
       <c r="H138">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I138" s="2" t="s">
         <v>16</v>
@@ -10698,7 +10698,7 @@
         <v>530</v>
       </c>
       <c r="H139">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="I139" s="2" t="s">
         <v>16</v>
@@ -10727,7 +10727,7 @@
         <v>534</v>
       </c>
       <c r="H140">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="I140" s="2" t="s">
         <v>16</v>
@@ -10756,7 +10756,7 @@
         <v>538</v>
       </c>
       <c r="H141">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="I141" s="2" t="s">
         <v>16</v>
@@ -10785,7 +10785,7 @@
         <v>542</v>
       </c>
       <c r="H142">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="I142" s="2" t="s">
         <v>16</v>
@@ -10814,7 +10814,7 @@
         <v>546</v>
       </c>
       <c r="H143">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I143" s="2" t="s">
         <v>16</v>
@@ -10843,7 +10843,7 @@
         <v>550</v>
       </c>
       <c r="H144">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I144" s="2" t="s">
         <v>16</v>
@@ -10872,7 +10872,7 @@
         <v>554</v>
       </c>
       <c r="H145">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="I145" s="2" t="s">
         <v>16</v>
@@ -10901,7 +10901,7 @@
         <v>558</v>
       </c>
       <c r="H146">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="I146" s="2" t="s">
         <v>16</v>
@@ -10930,7 +10930,7 @@
         <v>562</v>
       </c>
       <c r="H147">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="I147" s="2" t="s">
         <v>16</v>
@@ -10959,7 +10959,7 @@
         <v>566</v>
       </c>
       <c r="H148">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I148" s="2" t="s">
         <v>16</v>
@@ -10988,7 +10988,7 @@
         <v>570</v>
       </c>
       <c r="H149">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="I149" s="2" t="s">
         <v>16</v>
@@ -11017,7 +11017,7 @@
         <v>574</v>
       </c>
       <c r="H150">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I150" s="2" t="s">
         <v>16</v>
@@ -11046,7 +11046,7 @@
         <v>578</v>
       </c>
       <c r="H151">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="I151" s="2" t="s">
         <v>16</v>
@@ -11075,7 +11075,7 @@
         <v>583</v>
       </c>
       <c r="H152">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="I152" s="2" t="s">
         <v>16</v>
@@ -11104,7 +11104,7 @@
         <v>587</v>
       </c>
       <c r="H153">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="I153" s="2" t="s">
         <v>16</v>
@@ -11133,7 +11133,7 @@
         <v>591</v>
       </c>
       <c r="H154">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="I154" s="2" t="s">
         <v>16</v>
@@ -11162,7 +11162,7 @@
         <v>595</v>
       </c>
       <c r="H155">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="I155" s="2" t="s">
         <v>16</v>
@@ -11191,7 +11191,7 @@
         <v>599</v>
       </c>
       <c r="H156">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="I156" s="2" t="s">
         <v>16</v>
@@ -11220,7 +11220,7 @@
         <v>603</v>
       </c>
       <c r="H157">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="I157" s="2" t="s">
         <v>16</v>
@@ -11249,7 +11249,7 @@
         <v>607</v>
       </c>
       <c r="H158">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="I158" s="2" t="s">
         <v>16</v>
@@ -11278,7 +11278,7 @@
         <v>611</v>
       </c>
       <c r="H159">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="I159" s="2" t="s">
         <v>16</v>
@@ -11336,7 +11336,7 @@
         <v>619</v>
       </c>
       <c r="H161">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="I161" s="2" t="s">
         <v>16</v>
@@ -11365,7 +11365,7 @@
         <v>623</v>
       </c>
       <c r="H162">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I162" s="2" t="s">
         <v>16</v>
@@ -11394,7 +11394,7 @@
         <v>627</v>
       </c>
       <c r="H163">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="I163" s="2" t="s">
         <v>16</v>
@@ -11423,7 +11423,7 @@
         <v>631</v>
       </c>
       <c r="H164">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="I164" s="2" t="s">
         <v>16</v>
@@ -11452,7 +11452,7 @@
         <v>635</v>
       </c>
       <c r="H165">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I165" s="2" t="s">
         <v>16</v>
@@ -11481,7 +11481,7 @@
         <v>639</v>
       </c>
       <c r="H166">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="I166" s="2" t="s">
         <v>16</v>
@@ -11510,7 +11510,7 @@
         <v>643</v>
       </c>
       <c r="H167">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="I167" s="2" t="s">
         <v>16</v>
@@ -11539,7 +11539,7 @@
         <v>647</v>
       </c>
       <c r="H168">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I168" s="2" t="s">
         <v>16</v>
@@ -11568,7 +11568,7 @@
         <v>651</v>
       </c>
       <c r="H169">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="I169" s="2" t="s">
         <v>16</v>
@@ -11626,7 +11626,7 @@
         <v>659</v>
       </c>
       <c r="H171">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I171" s="2" t="s">
         <v>16</v>
@@ -11655,7 +11655,7 @@
         <v>664</v>
       </c>
       <c r="H172">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I172" s="2" t="s">
         <v>16</v>
@@ -11684,7 +11684,7 @@
         <v>668</v>
       </c>
       <c r="H173">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="I173" s="2" t="s">
         <v>16</v>
@@ -11713,7 +11713,7 @@
         <v>672</v>
       </c>
       <c r="H174">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="I174" s="2" t="s">
         <v>16</v>
@@ -11742,7 +11742,7 @@
         <v>676</v>
       </c>
       <c r="H175">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="I175" s="2" t="s">
         <v>16</v>
@@ -11771,7 +11771,7 @@
         <v>680</v>
       </c>
       <c r="H176">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="I176" s="2" t="s">
         <v>16</v>
@@ -11800,7 +11800,7 @@
         <v>684</v>
       </c>
       <c r="H177">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="I177" s="2" t="s">
         <v>16</v>
@@ -11829,7 +11829,7 @@
         <v>688</v>
       </c>
       <c r="H178">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="I178" s="2" t="s">
         <v>16</v>
@@ -11858,7 +11858,7 @@
         <v>692</v>
       </c>
       <c r="H179">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I179" s="2" t="s">
         <v>16</v>
@@ -11887,7 +11887,7 @@
         <v>696</v>
       </c>
       <c r="H180">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="I180" s="2" t="s">
         <v>16</v>
@@ -11945,7 +11945,7 @@
         <v>704</v>
       </c>
       <c r="H182">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="I182" s="2" t="s">
         <v>16</v>
@@ -11974,7 +11974,7 @@
         <v>708</v>
       </c>
       <c r="H183">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="I183" s="2" t="s">
         <v>16</v>
@@ -12003,7 +12003,7 @@
         <v>712</v>
       </c>
       <c r="H184">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="I184" s="2" t="s">
         <v>16</v>
@@ -12032,7 +12032,7 @@
         <v>716</v>
       </c>
       <c r="H185">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="I185" s="2" t="s">
         <v>16</v>
@@ -12061,7 +12061,7 @@
         <v>720</v>
       </c>
       <c r="H186">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="I186" s="2" t="s">
         <v>16</v>
@@ -12090,7 +12090,7 @@
         <v>724</v>
       </c>
       <c r="H187">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I187" s="2" t="s">
         <v>16</v>
@@ -12119,7 +12119,7 @@
         <v>728</v>
       </c>
       <c r="H188">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I188" s="2" t="s">
         <v>16</v>
@@ -12148,7 +12148,7 @@
         <v>732</v>
       </c>
       <c r="H189">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="I189" s="2" t="s">
         <v>16</v>
@@ -12177,7 +12177,7 @@
         <v>736</v>
       </c>
       <c r="H190">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="I190" s="2" t="s">
         <v>16</v>
@@ -12206,7 +12206,7 @@
         <v>740</v>
       </c>
       <c r="H191">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="I191" s="2" t="s">
         <v>16</v>
@@ -12235,7 +12235,7 @@
         <v>744</v>
       </c>
       <c r="H192">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="I192" s="2" t="s">
         <v>16</v>
@@ -12264,7 +12264,7 @@
         <v>748</v>
       </c>
       <c r="H193">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I193" s="2" t="s">
         <v>16</v>
@@ -12293,7 +12293,7 @@
         <v>752</v>
       </c>
       <c r="H194">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I194" s="2" t="s">
         <v>16</v>
@@ -12322,7 +12322,7 @@
         <v>756</v>
       </c>
       <c r="H195">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="I195" s="2" t="s">
         <v>16</v>
@@ -12351,7 +12351,7 @@
         <v>760</v>
       </c>
       <c r="H196">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="I196" s="2" t="s">
         <v>16</v>
@@ -12380,7 +12380,7 @@
         <v>764</v>
       </c>
       <c r="H197">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I197" s="2" t="s">
         <v>16</v>
@@ -12409,7 +12409,7 @@
         <v>768</v>
       </c>
       <c r="H198">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="I198" s="2" t="s">
         <v>16</v>
@@ -12438,7 +12438,7 @@
         <v>772</v>
       </c>
       <c r="H199">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I199" s="2" t="s">
         <v>16</v>
@@ -12467,7 +12467,7 @@
         <v>776</v>
       </c>
       <c r="H200">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="I200" s="2" t="s">
         <v>16</v>
@@ -12496,7 +12496,7 @@
         <v>780</v>
       </c>
       <c r="H201">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="I201" s="2" t="s">
         <v>16</v>
@@ -12525,7 +12525,7 @@
         <v>784</v>
       </c>
       <c r="H202">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I202" s="2" t="s">
         <v>16</v>
@@ -12554,7 +12554,7 @@
         <v>788</v>
       </c>
       <c r="H203">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="I203" s="2" t="s">
         <v>16</v>
@@ -12583,7 +12583,7 @@
         <v>792</v>
       </c>
       <c r="H204">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="I204" s="2" t="s">
         <v>16</v>
@@ -12612,7 +12612,7 @@
         <v>796</v>
       </c>
       <c r="H205">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="I205" s="2" t="s">
         <v>16</v>
@@ -12641,7 +12641,7 @@
         <v>800</v>
       </c>
       <c r="H206">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I206" s="2" t="s">
         <v>16</v>
@@ -12670,7 +12670,7 @@
         <v>804</v>
       </c>
       <c r="H207">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="I207" s="2" t="s">
         <v>16</v>
@@ -12699,7 +12699,7 @@
         <v>808</v>
       </c>
       <c r="H208">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I208" s="2" t="s">
         <v>16</v>
@@ -12728,7 +12728,7 @@
         <v>812</v>
       </c>
       <c r="H209">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="I209" s="2" t="s">
         <v>16</v>
@@ -12757,7 +12757,7 @@
         <v>816</v>
       </c>
       <c r="H210">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="I210" s="2" t="s">
         <v>16</v>
@@ -12786,7 +12786,7 @@
         <v>820</v>
       </c>
       <c r="H211">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="I211" s="2" t="s">
         <v>16</v>
@@ -12815,7 +12815,7 @@
         <v>825</v>
       </c>
       <c r="H212">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I212" s="2" t="s">
         <v>16</v>
@@ -12844,7 +12844,7 @@
         <v>829</v>
       </c>
       <c r="H213">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I213" s="2" t="s">
         <v>16</v>
@@ -12873,7 +12873,7 @@
         <v>833</v>
       </c>
       <c r="H214">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="I214" s="2" t="s">
         <v>16</v>
@@ -12902,7 +12902,7 @@
         <v>837</v>
       </c>
       <c r="H215">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="I215" s="2" t="s">
         <v>16</v>
@@ -12931,7 +12931,7 @@
         <v>841</v>
       </c>
       <c r="H216">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I216" s="2" t="s">
         <v>16</v>
@@ -12960,7 +12960,7 @@
         <v>845</v>
       </c>
       <c r="H217">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="I217" s="2" t="s">
         <v>16</v>
@@ -12989,7 +12989,7 @@
         <v>849</v>
       </c>
       <c r="H218">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="I218" s="2" t="s">
         <v>16</v>
@@ -13018,7 +13018,7 @@
         <v>853</v>
       </c>
       <c r="H219">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I219" s="2" t="s">
         <v>16</v>
@@ -13047,7 +13047,7 @@
         <v>857</v>
       </c>
       <c r="H220">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="I220" s="2" t="s">
         <v>16</v>
@@ -13076,7 +13076,7 @@
         <v>861</v>
       </c>
       <c r="H221">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="I221" s="2" t="s">
         <v>16</v>
@@ -13105,7 +13105,7 @@
         <v>865</v>
       </c>
       <c r="H222">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I222" s="2" t="s">
         <v>16</v>
@@ -13134,7 +13134,7 @@
         <v>869</v>
       </c>
       <c r="H223">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="I223" s="2" t="s">
         <v>16</v>
@@ -13163,7 +13163,7 @@
         <v>873</v>
       </c>
       <c r="H224">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I224" s="2" t="s">
         <v>16</v>
@@ -13192,7 +13192,7 @@
         <v>877</v>
       </c>
       <c r="H225">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="I225" s="2" t="s">
         <v>16</v>
@@ -13221,7 +13221,7 @@
         <v>881</v>
       </c>
       <c r="H226">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="I226" s="2" t="s">
         <v>16</v>
@@ -13250,7 +13250,7 @@
         <v>885</v>
       </c>
       <c r="H227">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="I227" s="2" t="s">
         <v>16</v>
@@ -13279,7 +13279,7 @@
         <v>889</v>
       </c>
       <c r="H228">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I228" s="2" t="s">
         <v>16</v>
@@ -13308,7 +13308,7 @@
         <v>893</v>
       </c>
       <c r="H229">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="I229" s="2" t="s">
         <v>16</v>
@@ -13337,7 +13337,7 @@
         <v>897</v>
       </c>
       <c r="H230">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="I230" s="2" t="s">
         <v>16</v>
@@ -13366,7 +13366,7 @@
         <v>901</v>
       </c>
       <c r="H231">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="I231" s="2" t="s">
         <v>16</v>
@@ -13395,7 +13395,7 @@
         <v>905</v>
       </c>
       <c r="H232">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="I232" s="2" t="s">
         <v>16</v>
@@ -13424,7 +13424,7 @@
         <v>909</v>
       </c>
       <c r="H233">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="I233" s="2" t="s">
         <v>16</v>
@@ -13453,7 +13453,7 @@
         <v>913</v>
       </c>
       <c r="H234">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="I234" s="2" t="s">
         <v>16</v>
@@ -13511,7 +13511,7 @@
         <v>921</v>
       </c>
       <c r="H236">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="I236" s="2" t="s">
         <v>16</v>
@@ -13540,7 +13540,7 @@
         <v>925</v>
       </c>
       <c r="H237">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I237" s="2" t="s">
         <v>16</v>
@@ -13569,7 +13569,7 @@
         <v>929</v>
       </c>
       <c r="H238">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="I238" s="2" t="s">
         <v>16</v>
@@ -13598,7 +13598,7 @@
         <v>933</v>
       </c>
       <c r="H239">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="I239" s="2" t="s">
         <v>16</v>
@@ -13627,7 +13627,7 @@
         <v>937</v>
       </c>
       <c r="H240">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="I240" s="2" t="s">
         <v>16</v>
@@ -13656,7 +13656,7 @@
         <v>941</v>
       </c>
       <c r="H241">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="I241" s="2" t="s">
         <v>16</v>
@@ -13685,7 +13685,7 @@
         <v>945</v>
       </c>
       <c r="H242">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="I242" s="2" t="s">
         <v>16</v>
@@ -13714,7 +13714,7 @@
         <v>949</v>
       </c>
       <c r="H243">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="I243" s="2" t="s">
         <v>16</v>
@@ -13743,7 +13743,7 @@
         <v>953</v>
       </c>
       <c r="H244">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I244" s="2" t="s">
         <v>16</v>
@@ -13772,7 +13772,7 @@
         <v>957</v>
       </c>
       <c r="H245">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="I245" s="2" t="s">
         <v>16</v>
@@ -13801,7 +13801,7 @@
         <v>961</v>
       </c>
       <c r="H246">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I246" s="2" t="s">
         <v>16</v>
@@ -13830,7 +13830,7 @@
         <v>965</v>
       </c>
       <c r="H247">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="I247" s="2" t="s">
         <v>16</v>
@@ -13859,7 +13859,7 @@
         <v>969</v>
       </c>
       <c r="H248">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I248" s="2" t="s">
         <v>16</v>
@@ -13888,7 +13888,7 @@
         <v>973</v>
       </c>
       <c r="H249">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I249" s="2" t="s">
         <v>16</v>
@@ -13917,7 +13917,7 @@
         <v>977</v>
       </c>
       <c r="H250">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="I250" s="2" t="s">
         <v>16</v>
@@ -13946,7 +13946,7 @@
         <v>981</v>
       </c>
       <c r="H251">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="I251" s="2" t="s">
         <v>16</v>
@@ -13975,7 +13975,7 @@
         <v>986</v>
       </c>
       <c r="H252">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="I252" s="2" t="s">
         <v>16</v>
@@ -14004,7 +14004,7 @@
         <v>990</v>
       </c>
       <c r="H253">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="I253" s="2" t="s">
         <v>16</v>
@@ -14033,7 +14033,7 @@
         <v>994</v>
       </c>
       <c r="H254">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="I254" s="2" t="s">
         <v>16</v>
@@ -14062,7 +14062,7 @@
         <v>998</v>
       </c>
       <c r="H255">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="I255" s="2" t="s">
         <v>16</v>
@@ -14091,7 +14091,7 @@
         <v>1002</v>
       </c>
       <c r="H256">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I256" s="2" t="s">
         <v>16</v>
@@ -14120,7 +14120,7 @@
         <v>1006</v>
       </c>
       <c r="H257">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="I257" s="2" t="s">
         <v>16</v>
@@ -14149,7 +14149,7 @@
         <v>1010</v>
       </c>
       <c r="H258">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="I258" s="2" t="s">
         <v>16</v>
@@ -14178,7 +14178,7 @@
         <v>1014</v>
       </c>
       <c r="H259">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="I259" s="2" t="s">
         <v>16</v>
@@ -14207,7 +14207,7 @@
         <v>1018</v>
       </c>
       <c r="H260">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="I260" s="2" t="s">
         <v>16</v>
@@ -14236,7 +14236,7 @@
         <v>1022</v>
       </c>
       <c r="H261">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="I261" s="2" t="s">
         <v>16</v>
@@ -14265,7 +14265,7 @@
         <v>1026</v>
       </c>
       <c r="H262">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="I262" s="2" t="s">
         <v>16</v>
@@ -14323,7 +14323,7 @@
         <v>1034</v>
       </c>
       <c r="H264">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I264" s="2" t="s">
         <v>16</v>
@@ -14352,7 +14352,7 @@
         <v>1038</v>
       </c>
       <c r="H265">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="I265" s="2" t="s">
         <v>16</v>
@@ -14381,7 +14381,7 @@
         <v>1042</v>
       </c>
       <c r="H266">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="I266" s="2" t="s">
         <v>16</v>
@@ -14410,7 +14410,7 @@
         <v>1046</v>
       </c>
       <c r="H267">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I267" s="2" t="s">
         <v>16</v>
@@ -14439,7 +14439,7 @@
         <v>1050</v>
       </c>
       <c r="H268">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="I268" s="2" t="s">
         <v>16</v>
@@ -14468,7 +14468,7 @@
         <v>1054</v>
       </c>
       <c r="H269">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="I269" s="2" t="s">
         <v>16</v>
@@ -14497,7 +14497,7 @@
         <v>1058</v>
       </c>
       <c r="H270">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I270" s="2" t="s">
         <v>16</v>
@@ -14526,7 +14526,7 @@
         <v>1062</v>
       </c>
       <c r="H271">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I271" s="2" t="s">
         <v>16</v>
@@ -14555,7 +14555,7 @@
         <v>1067</v>
       </c>
       <c r="H272">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="I272" s="2" t="s">
         <v>16</v>
@@ -14584,7 +14584,7 @@
         <v>1071</v>
       </c>
       <c r="H273">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="I273" s="2" t="s">
         <v>16</v>
@@ -14613,7 +14613,7 @@
         <v>1075</v>
       </c>
       <c r="H274">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="I274" s="2" t="s">
         <v>16</v>
@@ -14642,7 +14642,7 @@
         <v>1079</v>
       </c>
       <c r="H275">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="I275" s="2" t="s">
         <v>16</v>
@@ -14671,7 +14671,7 @@
         <v>1083</v>
       </c>
       <c r="H276">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="I276" s="2" t="s">
         <v>16</v>
@@ -14700,7 +14700,7 @@
         <v>1087</v>
       </c>
       <c r="H277">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="I277" s="2" t="s">
         <v>16</v>
@@ -14729,7 +14729,7 @@
         <v>1091</v>
       </c>
       <c r="H278">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="I278" s="2" t="s">
         <v>16</v>
@@ -14758,7 +14758,7 @@
         <v>1095</v>
       </c>
       <c r="H279">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="I279" s="2" t="s">
         <v>16</v>
@@ -14787,7 +14787,7 @@
         <v>1099</v>
       </c>
       <c r="H280">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="I280" s="2" t="s">
         <v>16</v>
@@ -14816,7 +14816,7 @@
         <v>1103</v>
       </c>
       <c r="H281">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I281" s="2" t="s">
         <v>16</v>
@@ -14845,7 +14845,7 @@
         <v>1107</v>
       </c>
       <c r="H282">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="I282" s="2" t="s">
         <v>16</v>
@@ -14874,7 +14874,7 @@
         <v>1111</v>
       </c>
       <c r="H283">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="I283" s="2" t="s">
         <v>16</v>
@@ -14903,7 +14903,7 @@
         <v>1115</v>
       </c>
       <c r="H284">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I284" s="2" t="s">
         <v>16</v>
@@ -14932,7 +14932,7 @@
         <v>1119</v>
       </c>
       <c r="H285">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="I285" s="2" t="s">
         <v>16</v>
@@ -14961,7 +14961,7 @@
         <v>1123</v>
       </c>
       <c r="H286">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="I286" s="2" t="s">
         <v>16</v>
@@ -14990,7 +14990,7 @@
         <v>1127</v>
       </c>
       <c r="H287">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="I287" s="2" t="s">
         <v>16</v>
@@ -15019,7 +15019,7 @@
         <v>1131</v>
       </c>
       <c r="H288">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="I288" s="2" t="s">
         <v>16</v>
@@ -15048,7 +15048,7 @@
         <v>1135</v>
       </c>
       <c r="H289">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="I289" s="2" t="s">
         <v>16</v>
@@ -15077,7 +15077,7 @@
         <v>1139</v>
       </c>
       <c r="H290">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I290" s="2" t="s">
         <v>16</v>
@@ -15106,7 +15106,7 @@
         <v>1143</v>
       </c>
       <c r="H291">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="I291" s="2" t="s">
         <v>16</v>
@@ -15135,7 +15135,7 @@
         <v>1148</v>
       </c>
       <c r="H292">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="I292" s="2" t="s">
         <v>16</v>
@@ -15164,7 +15164,7 @@
         <v>1152</v>
       </c>
       <c r="H293">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="I293" s="2" t="s">
         <v>16</v>
@@ -15193,7 +15193,7 @@
         <v>1156</v>
       </c>
       <c r="H294">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I294" s="2" t="s">
         <v>16</v>
@@ -15222,7 +15222,7 @@
         <v>1160</v>
       </c>
       <c r="H295">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="I295" s="2" t="s">
         <v>16</v>
@@ -15251,7 +15251,7 @@
         <v>1164</v>
       </c>
       <c r="H296">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="I296" s="2" t="s">
         <v>16</v>
@@ -15280,7 +15280,7 @@
         <v>1168</v>
       </c>
       <c r="H297">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="I297" s="2" t="s">
         <v>16</v>
@@ -15309,7 +15309,7 @@
         <v>1172</v>
       </c>
       <c r="H298">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="I298" s="2" t="s">
         <v>16</v>
@@ -15338,7 +15338,7 @@
         <v>1176</v>
       </c>
       <c r="H299">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="I299" s="2" t="s">
         <v>16</v>
@@ -15367,7 +15367,7 @@
         <v>1180</v>
       </c>
       <c r="H300">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I300" s="2" t="s">
         <v>16</v>
@@ -15396,7 +15396,7 @@
         <v>1184</v>
       </c>
       <c r="H301">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="I301" s="2" t="s">
         <v>16</v>
@@ -15425,7 +15425,7 @@
         <v>1188</v>
       </c>
       <c r="H302">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="I302" s="2" t="s">
         <v>16</v>
@@ -15454,7 +15454,7 @@
         <v>1192</v>
       </c>
       <c r="H303">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="I303" s="2" t="s">
         <v>16</v>
@@ -15483,7 +15483,7 @@
         <v>1196</v>
       </c>
       <c r="H304">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="I304" s="2" t="s">
         <v>16</v>
@@ -15512,7 +15512,7 @@
         <v>1200</v>
       </c>
       <c r="H305">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="I305" s="2" t="s">
         <v>16</v>
@@ -15541,7 +15541,7 @@
         <v>1204</v>
       </c>
       <c r="H306">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="I306" s="2" t="s">
         <v>16</v>
@@ -15570,7 +15570,7 @@
         <v>1208</v>
       </c>
       <c r="H307">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I307" s="2" t="s">
         <v>16</v>
@@ -15599,7 +15599,7 @@
         <v>1212</v>
       </c>
       <c r="H308">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="I308" s="2" t="s">
         <v>16</v>
@@ -15628,7 +15628,7 @@
         <v>1216</v>
       </c>
       <c r="H309">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="I309" s="2" t="s">
         <v>16</v>
@@ -15657,7 +15657,7 @@
         <v>1220</v>
       </c>
       <c r="H310">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="I310" s="2" t="s">
         <v>16</v>
@@ -15686,7 +15686,7 @@
         <v>1224</v>
       </c>
       <c r="H311">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="I311" s="2" t="s">
         <v>16</v>
@@ -15715,7 +15715,7 @@
         <v>1228</v>
       </c>
       <c r="H312">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="I312" s="2" t="s">
         <v>16</v>
@@ -15744,7 +15744,7 @@
         <v>1232</v>
       </c>
       <c r="H313">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="I313" s="2" t="s">
         <v>16</v>
@@ -15773,7 +15773,7 @@
         <v>1236</v>
       </c>
       <c r="H314">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I314" s="2" t="s">
         <v>16</v>
@@ -15802,7 +15802,7 @@
         <v>1240</v>
       </c>
       <c r="H315">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="I315" s="2" t="s">
         <v>16</v>
@@ -15831,7 +15831,7 @@
         <v>1244</v>
       </c>
       <c r="H316">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="I316" s="2" t="s">
         <v>16</v>
@@ -15860,7 +15860,7 @@
         <v>1248</v>
       </c>
       <c r="H317">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="I317" s="2" t="s">
         <v>16</v>
@@ -15889,7 +15889,7 @@
         <v>1252</v>
       </c>
       <c r="H318">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="I318" s="2" t="s">
         <v>16</v>
@@ -15918,7 +15918,7 @@
         <v>1256</v>
       </c>
       <c r="H319">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="I319" s="2" t="s">
         <v>16</v>
@@ -15947,7 +15947,7 @@
         <v>1260</v>
       </c>
       <c r="H320">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I320" s="2" t="s">
         <v>16</v>
@@ -15976,7 +15976,7 @@
         <v>1264</v>
       </c>
       <c r="H321">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="I321" s="2" t="s">
         <v>16</v>
@@ -16005,7 +16005,7 @@
         <v>1268</v>
       </c>
       <c r="H322">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="I322" s="2" t="s">
         <v>16</v>
@@ -16034,7 +16034,7 @@
         <v>1272</v>
       </c>
       <c r="H323">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I323" s="2" t="s">
         <v>16</v>
@@ -16063,7 +16063,7 @@
         <v>1276</v>
       </c>
       <c r="H324">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="I324" s="2" t="s">
         <v>16</v>
@@ -16092,7 +16092,7 @@
         <v>1280</v>
       </c>
       <c r="H325">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="I325" s="2" t="s">
         <v>16</v>
@@ -16121,7 +16121,7 @@
         <v>1284</v>
       </c>
       <c r="H326">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="I326" s="2" t="s">
         <v>16</v>
@@ -16150,7 +16150,7 @@
         <v>1288</v>
       </c>
       <c r="H327">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="I327" s="2" t="s">
         <v>16</v>
@@ -16179,7 +16179,7 @@
         <v>1292</v>
       </c>
       <c r="H328">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="I328" s="2" t="s">
         <v>16</v>
@@ -16208,7 +16208,7 @@
         <v>1296</v>
       </c>
       <c r="H329">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="I329" s="2" t="s">
         <v>16</v>
@@ -16237,7 +16237,7 @@
         <v>1300</v>
       </c>
       <c r="H330">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I330" s="2" t="s">
         <v>16</v>
@@ -16266,7 +16266,7 @@
         <v>1304</v>
       </c>
       <c r="H331">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="I331" s="2" t="s">
         <v>16</v>
@@ -16295,7 +16295,7 @@
         <v>1309</v>
       </c>
       <c r="H332">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I332" s="2" t="s">
         <v>16</v>
@@ -16324,7 +16324,7 @@
         <v>1313</v>
       </c>
       <c r="H333">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="I333" s="2" t="s">
         <v>16</v>
@@ -16353,7 +16353,7 @@
         <v>1317</v>
       </c>
       <c r="H334">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="I334" s="2" t="s">
         <v>16</v>
@@ -16382,7 +16382,7 @@
         <v>1321</v>
       </c>
       <c r="H335">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="I335" s="2" t="s">
         <v>16</v>
@@ -16411,7 +16411,7 @@
         <v>1325</v>
       </c>
       <c r="H336">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="I336" s="2" t="s">
         <v>16</v>
@@ -16440,7 +16440,7 @@
         <v>1329</v>
       </c>
       <c r="H337">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="I337" s="2" t="s">
         <v>16</v>
@@ -16469,7 +16469,7 @@
         <v>1333</v>
       </c>
       <c r="H338">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I338" s="2" t="s">
         <v>16</v>
@@ -16498,7 +16498,7 @@
         <v>1337</v>
       </c>
       <c r="H339">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="I339" s="2" t="s">
         <v>16</v>
@@ -16527,7 +16527,7 @@
         <v>1341</v>
       </c>
       <c r="H340">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I340" s="2" t="s">
         <v>16</v>
@@ -16556,7 +16556,7 @@
         <v>1345</v>
       </c>
       <c r="H341">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="I341" s="2" t="s">
         <v>16</v>
@@ -16585,7 +16585,7 @@
         <v>1349</v>
       </c>
       <c r="H342">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="I342" s="2" t="s">
         <v>16</v>
@@ -16614,7 +16614,7 @@
         <v>1353</v>
       </c>
       <c r="H343">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="I343" s="2" t="s">
         <v>16</v>
@@ -16643,7 +16643,7 @@
         <v>1357</v>
       </c>
       <c r="H344">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="I344" s="2" t="s">
         <v>16</v>
@@ -16672,7 +16672,7 @@
         <v>1361</v>
       </c>
       <c r="H345">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="I345" s="2" t="s">
         <v>16</v>
@@ -16701,7 +16701,7 @@
         <v>1365</v>
       </c>
       <c r="H346">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I346" s="2" t="s">
         <v>16</v>
@@ -16730,7 +16730,7 @@
         <v>1369</v>
       </c>
       <c r="H347">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I347" s="2" t="s">
         <v>16</v>
@@ -16759,7 +16759,7 @@
         <v>1373</v>
       </c>
       <c r="H348">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="I348" s="2" t="s">
         <v>16</v>
@@ -16788,7 +16788,7 @@
         <v>1377</v>
       </c>
       <c r="H349">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="I349" s="2" t="s">
         <v>16</v>
@@ -16817,7 +16817,7 @@
         <v>1381</v>
       </c>
       <c r="H350">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I350" s="2" t="s">
         <v>16</v>
@@ -16846,7 +16846,7 @@
         <v>1385</v>
       </c>
       <c r="H351">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I351" s="2" t="s">
         <v>16</v>
@@ -16875,7 +16875,7 @@
         <v>1390</v>
       </c>
       <c r="H352">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I352" s="2" t="s">
         <v>16</v>
@@ -16904,7 +16904,7 @@
         <v>1394</v>
       </c>
       <c r="H353">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="I353" s="2" t="s">
         <v>16</v>
@@ -16933,7 +16933,7 @@
         <v>1398</v>
       </c>
       <c r="H354">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="I354" s="2" t="s">
         <v>16</v>
@@ -16962,7 +16962,7 @@
         <v>1402</v>
       </c>
       <c r="H355">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="I355" s="2" t="s">
         <v>16</v>
@@ -16991,7 +16991,7 @@
         <v>1406</v>
       </c>
       <c r="H356">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I356" s="2" t="s">
         <v>16</v>
@@ -17020,7 +17020,7 @@
         <v>1410</v>
       </c>
       <c r="H357">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="I357" s="2" t="s">
         <v>16</v>
@@ -17049,7 +17049,7 @@
         <v>1414</v>
       </c>
       <c r="H358">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="I358" s="2" t="s">
         <v>16</v>
@@ -17107,7 +17107,7 @@
         <v>1422</v>
       </c>
       <c r="H360">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="I360" s="2" t="s">
         <v>16</v>
@@ -17136,7 +17136,7 @@
         <v>1426</v>
       </c>
       <c r="H361">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="I361" s="2" t="s">
         <v>16</v>
@@ -17165,7 +17165,7 @@
         <v>1430</v>
       </c>
       <c r="H362">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="I362" s="2" t="s">
         <v>16</v>
@@ -17194,7 +17194,7 @@
         <v>1434</v>
       </c>
       <c r="H363">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="I363" s="2" t="s">
         <v>16</v>
@@ -17223,7 +17223,7 @@
         <v>1438</v>
       </c>
       <c r="H364">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="I364" s="2" t="s">
         <v>16</v>
@@ -17252,7 +17252,7 @@
         <v>1442</v>
       </c>
       <c r="H365">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="I365" s="2" t="s">
         <v>16</v>
@@ -17281,7 +17281,7 @@
         <v>1446</v>
       </c>
       <c r="H366">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="I366" s="2" t="s">
         <v>16</v>
@@ -17310,7 +17310,7 @@
         <v>1450</v>
       </c>
       <c r="H367">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I367" s="2" t="s">
         <v>16</v>
@@ -17339,7 +17339,7 @@
         <v>1454</v>
       </c>
       <c r="H368">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="I368" s="2" t="s">
         <v>16</v>
@@ -17368,7 +17368,7 @@
         <v>1458</v>
       </c>
       <c r="H369">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="I369" s="2" t="s">
         <v>16</v>
@@ -17397,7 +17397,7 @@
         <v>1462</v>
       </c>
       <c r="H370">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I370" s="2" t="s">
         <v>16</v>
@@ -17426,7 +17426,7 @@
         <v>1466</v>
       </c>
       <c r="H371">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="I371" s="2" t="s">
         <v>16</v>
@@ -17455,7 +17455,7 @@
         <v>1471</v>
       </c>
       <c r="H372">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="I372" s="2" t="s">
         <v>16</v>
@@ -17484,7 +17484,7 @@
         <v>1475</v>
       </c>
       <c r="H373">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="I373" s="2" t="s">
         <v>16</v>
@@ -17513,7 +17513,7 @@
         <v>1479</v>
       </c>
       <c r="H374">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="I374" s="2" t="s">
         <v>16</v>
@@ -17542,7 +17542,7 @@
         <v>1483</v>
       </c>
       <c r="H375">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="I375" s="2" t="s">
         <v>16</v>
@@ -17600,7 +17600,7 @@
         <v>1491</v>
       </c>
       <c r="H377">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="I377" s="2" t="s">
         <v>16</v>
@@ -17629,7 +17629,7 @@
         <v>1495</v>
       </c>
       <c r="H378">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I378" s="2" t="s">
         <v>16</v>
@@ -17658,7 +17658,7 @@
         <v>1499</v>
       </c>
       <c r="H379">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I379" s="2" t="s">
         <v>16</v>
@@ -17687,7 +17687,7 @@
         <v>1503</v>
       </c>
       <c r="H380">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I380" s="2" t="s">
         <v>16</v>
@@ -17716,7 +17716,7 @@
         <v>1507</v>
       </c>
       <c r="H381">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="I381" s="2" t="s">
         <v>16</v>
@@ -17745,7 +17745,7 @@
         <v>1511</v>
       </c>
       <c r="H382">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="I382" s="2" t="s">
         <v>16</v>
@@ -17774,7 +17774,7 @@
         <v>1515</v>
       </c>
       <c r="H383">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="I383" s="2" t="s">
         <v>16</v>
@@ -17803,7 +17803,7 @@
         <v>1519</v>
       </c>
       <c r="H384">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="I384" s="2" t="s">
         <v>16</v>
@@ -17832,7 +17832,7 @@
         <v>1523</v>
       </c>
       <c r="H385">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="I385" s="2" t="s">
         <v>16</v>
@@ -17861,7 +17861,7 @@
         <v>1527</v>
       </c>
       <c r="H386">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="I386" s="2" t="s">
         <v>16</v>
@@ -17890,7 +17890,7 @@
         <v>1531</v>
       </c>
       <c r="H387">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="I387" s="2" t="s">
         <v>16</v>
@@ -17919,7 +17919,7 @@
         <v>1535</v>
       </c>
       <c r="H388">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="I388" s="2" t="s">
         <v>16</v>
@@ -17948,7 +17948,7 @@
         <v>1539</v>
       </c>
       <c r="H389">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I389" s="2" t="s">
         <v>16</v>
@@ -17977,7 +17977,7 @@
         <v>1543</v>
       </c>
       <c r="H390">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="I390" s="2" t="s">
         <v>16</v>
@@ -18006,7 +18006,7 @@
         <v>1547</v>
       </c>
       <c r="H391">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="I391" s="2" t="s">
         <v>16</v>
@@ -18035,7 +18035,7 @@
         <v>1552</v>
       </c>
       <c r="H392">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="I392" s="2" t="s">
         <v>16</v>
@@ -18093,7 +18093,7 @@
         <v>1560</v>
       </c>
       <c r="H394">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="I394" s="2" t="s">
         <v>16</v>
@@ -18122,7 +18122,7 @@
         <v>1564</v>
       </c>
       <c r="H395">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="I395" s="2" t="s">
         <v>16</v>
@@ -18151,7 +18151,7 @@
         <v>1568</v>
       </c>
       <c r="H396">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="I396" s="2" t="s">
         <v>16</v>
@@ -18180,7 +18180,7 @@
         <v>1572</v>
       </c>
       <c r="H397">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="I397" s="2" t="s">
         <v>16</v>
@@ -18209,7 +18209,7 @@
         <v>1576</v>
       </c>
       <c r="H398">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I398" s="2" t="s">
         <v>16</v>
@@ -18238,7 +18238,7 @@
         <v>1580</v>
       </c>
       <c r="H399">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="I399" s="2" t="s">
         <v>16</v>
@@ -18267,7 +18267,7 @@
         <v>1584</v>
       </c>
       <c r="H400">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="I400" s="2" t="s">
         <v>16</v>
@@ -18296,7 +18296,7 @@
         <v>1588</v>
       </c>
       <c r="H401">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="I401" s="2" t="s">
         <v>16</v>
@@ -18325,7 +18325,7 @@
         <v>1592</v>
       </c>
       <c r="H402">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="I402" s="2" t="s">
         <v>16</v>
@@ -18354,7 +18354,7 @@
         <v>1596</v>
       </c>
       <c r="H403">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="I403" s="2" t="s">
         <v>16</v>
@@ -18383,7 +18383,7 @@
         <v>1600</v>
       </c>
       <c r="H404">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="I404" s="2" t="s">
         <v>16</v>
@@ -18412,7 +18412,7 @@
         <v>1604</v>
       </c>
       <c r="H405">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="I405" s="2" t="s">
         <v>16</v>
@@ -18441,7 +18441,7 @@
         <v>1608</v>
       </c>
       <c r="H406">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="I406" s="2" t="s">
         <v>16</v>
@@ -18470,7 +18470,7 @@
         <v>1612</v>
       </c>
       <c r="H407">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="I407" s="2" t="s">
         <v>16</v>
@@ -18499,7 +18499,7 @@
         <v>1616</v>
       </c>
       <c r="H408">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="I408" s="2" t="s">
         <v>16</v>
@@ -18528,7 +18528,7 @@
         <v>1620</v>
       </c>
       <c r="H409">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="I409" s="2" t="s">
         <v>16</v>
@@ -18557,7 +18557,7 @@
         <v>1624</v>
       </c>
       <c r="H410">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="I410" s="2" t="s">
         <v>16</v>
@@ -18586,7 +18586,7 @@
         <v>1628</v>
       </c>
       <c r="H411">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I411" s="2" t="s">
         <v>16</v>
@@ -18615,7 +18615,7 @@
         <v>1633</v>
       </c>
       <c r="H412">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="I412" s="2" t="s">
         <v>16</v>
@@ -18644,7 +18644,7 @@
         <v>1637</v>
       </c>
       <c r="H413">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="I413" s="2" t="s">
         <v>16</v>
@@ -18673,7 +18673,7 @@
         <v>1641</v>
       </c>
       <c r="H414">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="I414" s="2" t="s">
         <v>16</v>
@@ -18702,7 +18702,7 @@
         <v>1645</v>
       </c>
       <c r="H415">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="I415" s="2" t="s">
         <v>16</v>
@@ -18731,7 +18731,7 @@
         <v>1649</v>
       </c>
       <c r="H416">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I416" s="2" t="s">
         <v>16</v>
@@ -18760,7 +18760,7 @@
         <v>1653</v>
       </c>
       <c r="H417">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I417" s="2" t="s">
         <v>16</v>
@@ -18789,7 +18789,7 @@
         <v>1657</v>
       </c>
       <c r="H418">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I418" s="2" t="s">
         <v>16</v>
@@ -18818,7 +18818,7 @@
         <v>1661</v>
       </c>
       <c r="H419">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="I419" s="2" t="s">
         <v>16</v>
@@ -18847,7 +18847,7 @@
         <v>1665</v>
       </c>
       <c r="H420">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="I420" s="2" t="s">
         <v>16</v>
@@ -18876,7 +18876,7 @@
         <v>1669</v>
       </c>
       <c r="H421">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="I421" s="2" t="s">
         <v>16</v>
@@ -18905,7 +18905,7 @@
         <v>1674</v>
       </c>
       <c r="H422">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I422" s="2" t="s">
         <v>16</v>
@@ -18934,7 +18934,7 @@
         <v>1678</v>
       </c>
       <c r="H423">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="I423" s="2" t="s">
         <v>16</v>
@@ -18963,7 +18963,7 @@
         <v>1682</v>
       </c>
       <c r="H424">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="I424" s="2" t="s">
         <v>16</v>
@@ -18992,7 +18992,7 @@
         <v>1686</v>
       </c>
       <c r="H425">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I425" s="2" t="s">
         <v>16</v>
@@ -19021,7 +19021,7 @@
         <v>1690</v>
       </c>
       <c r="H426">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="I426" s="2" t="s">
         <v>16</v>
@@ -19050,7 +19050,7 @@
         <v>1694</v>
       </c>
       <c r="H427">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="I427" s="2" t="s">
         <v>16</v>
@@ -19079,7 +19079,7 @@
         <v>1698</v>
       </c>
       <c r="H428">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="I428" s="2" t="s">
         <v>16</v>
@@ -19108,7 +19108,7 @@
         <v>1702</v>
       </c>
       <c r="H429">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="I429" s="2" t="s">
         <v>16</v>
@@ -19137,7 +19137,7 @@
         <v>1706</v>
       </c>
       <c r="H430">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="I430" s="2" t="s">
         <v>16</v>
@@ -19166,7 +19166,7 @@
         <v>1710</v>
       </c>
       <c r="H431">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="I431" s="2" t="s">
         <v>16</v>
@@ -19195,7 +19195,7 @@
         <v>1714</v>
       </c>
       <c r="H432">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="I432" s="2" t="s">
         <v>16</v>
@@ -19224,7 +19224,7 @@
         <v>1718</v>
       </c>
       <c r="H433">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="I433" s="2" t="s">
         <v>16</v>
@@ -19253,7 +19253,7 @@
         <v>1722</v>
       </c>
       <c r="H434">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="I434" s="2" t="s">
         <v>16</v>
@@ -19282,7 +19282,7 @@
         <v>1726</v>
       </c>
       <c r="H435">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="I435" s="2" t="s">
         <v>16</v>
@@ -19311,7 +19311,7 @@
         <v>1730</v>
       </c>
       <c r="H436">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="I436" s="2" t="s">
         <v>16</v>
@@ -19340,7 +19340,7 @@
         <v>1734</v>
       </c>
       <c r="H437">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="I437" s="2" t="s">
         <v>16</v>
@@ -19369,7 +19369,7 @@
         <v>1738</v>
       </c>
       <c r="H438">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="I438" s="2" t="s">
         <v>16</v>
@@ -19398,7 +19398,7 @@
         <v>1742</v>
       </c>
       <c r="H439">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I439" s="2" t="s">
         <v>16</v>
@@ -19427,7 +19427,7 @@
         <v>1746</v>
       </c>
       <c r="H440">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I440" s="2" t="s">
         <v>16</v>
@@ -19456,7 +19456,7 @@
         <v>1750</v>
       </c>
       <c r="H441">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I441" s="2" t="s">
         <v>16</v>
@@ -19485,7 +19485,7 @@
         <v>1755</v>
       </c>
       <c r="H442">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="I442" s="2" t="s">
         <v>16</v>
@@ -19514,7 +19514,7 @@
         <v>1759</v>
       </c>
       <c r="H443">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="I443" s="2" t="s">
         <v>16</v>
@@ -19572,7 +19572,7 @@
         <v>1767</v>
       </c>
       <c r="H445">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="I445" s="2" t="s">
         <v>16</v>
@@ -19601,7 +19601,7 @@
         <v>1771</v>
       </c>
       <c r="H446">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="I446" s="2" t="s">
         <v>16</v>
@@ -19630,7 +19630,7 @@
         <v>1775</v>
       </c>
       <c r="H447">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I447" s="2" t="s">
         <v>16</v>
@@ -19659,7 +19659,7 @@
         <v>1779</v>
       </c>
       <c r="H448">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="I448" s="2" t="s">
         <v>16</v>
@@ -19688,7 +19688,7 @@
         <v>1783</v>
       </c>
       <c r="H449">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="I449" s="2" t="s">
         <v>16</v>
@@ -19717,7 +19717,7 @@
         <v>1787</v>
       </c>
       <c r="H450">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="I450" s="2" t="s">
         <v>16</v>
@@ -19746,7 +19746,7 @@
         <v>1791</v>
       </c>
       <c r="H451">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I451" s="2" t="s">
         <v>16</v>
@@ -19775,7 +19775,7 @@
         <v>1796</v>
       </c>
       <c r="H452">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I452" s="2" t="s">
         <v>16</v>
@@ -19804,7 +19804,7 @@
         <v>1800</v>
       </c>
       <c r="H453">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="I453" s="2" t="s">
         <v>16</v>
@@ -19833,7 +19833,7 @@
         <v>1804</v>
       </c>
       <c r="H454">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="I454" s="2" t="s">
         <v>16</v>
@@ -19862,7 +19862,7 @@
         <v>1808</v>
       </c>
       <c r="H455">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="I455" s="2" t="s">
         <v>16</v>
@@ -19891,7 +19891,7 @@
         <v>1812</v>
       </c>
       <c r="H456">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="I456" s="2" t="s">
         <v>16</v>
@@ -19920,7 +19920,7 @@
         <v>1816</v>
       </c>
       <c r="H457">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="I457" s="2" t="s">
         <v>16</v>
@@ -19949,7 +19949,7 @@
         <v>1820</v>
       </c>
       <c r="H458">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="I458" s="2" t="s">
         <v>16</v>
@@ -19978,7 +19978,7 @@
         <v>1824</v>
       </c>
       <c r="H459">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I459" s="2" t="s">
         <v>16</v>
@@ -20007,7 +20007,7 @@
         <v>1828</v>
       </c>
       <c r="H460">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="I460" s="2" t="s">
         <v>16</v>
@@ -20036,7 +20036,7 @@
         <v>1832</v>
       </c>
       <c r="H461">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="I461" s="2" t="s">
         <v>16</v>
@@ -20065,7 +20065,7 @@
         <v>1836</v>
       </c>
       <c r="H462">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="I462" s="2" t="s">
         <v>16</v>
@@ -20094,7 +20094,7 @@
         <v>1840</v>
       </c>
       <c r="H463">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="I463" s="2" t="s">
         <v>16</v>
@@ -20123,7 +20123,7 @@
         <v>1844</v>
       </c>
       <c r="H464">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="I464" s="2" t="s">
         <v>16</v>
@@ -20152,7 +20152,7 @@
         <v>1848</v>
       </c>
       <c r="H465">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="I465" s="2" t="s">
         <v>16</v>
@@ -20181,7 +20181,7 @@
         <v>1852</v>
       </c>
       <c r="H466">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I466" s="2" t="s">
         <v>16</v>
@@ -20210,7 +20210,7 @@
         <v>1856</v>
       </c>
       <c r="H467">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="I467" s="2" t="s">
         <v>16</v>
@@ -20239,7 +20239,7 @@
         <v>1860</v>
       </c>
       <c r="H468">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I468" s="2" t="s">
         <v>16</v>
@@ -20268,7 +20268,7 @@
         <v>1864</v>
       </c>
       <c r="H469">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="I469" s="2" t="s">
         <v>16</v>
@@ -20297,7 +20297,7 @@
         <v>1868</v>
       </c>
       <c r="H470">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="I470" s="2" t="s">
         <v>16</v>
@@ -20326,7 +20326,7 @@
         <v>1872</v>
       </c>
       <c r="H471">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="I471" s="2" t="s">
         <v>16</v>
@@ -20355,7 +20355,7 @@
         <v>1877</v>
       </c>
       <c r="H472">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I472" s="2" t="s">
         <v>16</v>
@@ -20384,7 +20384,7 @@
         <v>1881</v>
       </c>
       <c r="H473">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="I473" s="2" t="s">
         <v>16</v>
@@ -20413,7 +20413,7 @@
         <v>1885</v>
       </c>
       <c r="H474">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I474" s="2" t="s">
         <v>16</v>
@@ -20442,7 +20442,7 @@
         <v>1889</v>
       </c>
       <c r="H475">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="I475" s="2" t="s">
         <v>16</v>
@@ -20471,7 +20471,7 @@
         <v>1893</v>
       </c>
       <c r="H476">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="I476" s="2" t="s">
         <v>16</v>
@@ -20500,7 +20500,7 @@
         <v>1897</v>
       </c>
       <c r="H477">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I477" s="2" t="s">
         <v>16</v>
@@ -20529,7 +20529,7 @@
         <v>1901</v>
       </c>
       <c r="H478">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I478" s="2" t="s">
         <v>16</v>
@@ -20558,7 +20558,7 @@
         <v>1905</v>
       </c>
       <c r="H479">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I479" s="2" t="s">
         <v>16</v>
@@ -20587,7 +20587,7 @@
         <v>1909</v>
       </c>
       <c r="H480">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="I480" s="2" t="s">
         <v>16</v>
@@ -20616,7 +20616,7 @@
         <v>1913</v>
       </c>
       <c r="H481">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="I481" s="2" t="s">
         <v>16</v>
@@ -20645,7 +20645,7 @@
         <v>1917</v>
       </c>
       <c r="H482">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="I482" s="2" t="s">
         <v>16</v>
@@ -20674,7 +20674,7 @@
         <v>1921</v>
       </c>
       <c r="H483">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="I483" s="2" t="s">
         <v>16</v>
@@ -20703,7 +20703,7 @@
         <v>1925</v>
       </c>
       <c r="H484">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I484" s="2" t="s">
         <v>16</v>
@@ -20732,7 +20732,7 @@
         <v>1929</v>
       </c>
       <c r="H485">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="I485" s="2" t="s">
         <v>16</v>
@@ -20761,7 +20761,7 @@
         <v>1933</v>
       </c>
       <c r="H486">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I486" s="2" t="s">
         <v>16</v>
@@ -20790,7 +20790,7 @@
         <v>1937</v>
       </c>
       <c r="H487">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="I487" s="2" t="s">
         <v>16</v>
@@ -20819,7 +20819,7 @@
         <v>1941</v>
       </c>
       <c r="H488">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="I488" s="2" t="s">
         <v>16</v>
@@ -20848,7 +20848,7 @@
         <v>1945</v>
       </c>
       <c r="H489">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="I489" s="2" t="s">
         <v>16</v>
@@ -20877,7 +20877,7 @@
         <v>1949</v>
       </c>
       <c r="H490">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="I490" s="2" t="s">
         <v>16</v>
@@ -20906,7 +20906,7 @@
         <v>1953</v>
       </c>
       <c r="H491">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="I491" s="2" t="s">
         <v>16</v>
@@ -20935,7 +20935,7 @@
         <v>1957</v>
       </c>
       <c r="H492">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I492" s="2" t="s">
         <v>16</v>
@@ -20964,7 +20964,7 @@
         <v>1961</v>
       </c>
       <c r="H493">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I493" s="2" t="s">
         <v>16</v>
@@ -20993,7 +20993,7 @@
         <v>1965</v>
       </c>
       <c r="H494">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I494" s="2" t="s">
         <v>16</v>
@@ -21022,7 +21022,7 @@
         <v>1969</v>
       </c>
       <c r="H495">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="I495" s="2" t="s">
         <v>16</v>
@@ -21051,7 +21051,7 @@
         <v>1973</v>
       </c>
       <c r="H496">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="I496" s="2" t="s">
         <v>16</v>
@@ -21080,7 +21080,7 @@
         <v>1977</v>
       </c>
       <c r="H497">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="I497" s="2" t="s">
         <v>16</v>
@@ -21109,7 +21109,7 @@
         <v>1981</v>
       </c>
       <c r="H498">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="I498" s="2" t="s">
         <v>16</v>
@@ -21138,7 +21138,7 @@
         <v>1985</v>
       </c>
       <c r="H499">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I499" s="2" t="s">
         <v>16</v>
@@ -21167,7 +21167,7 @@
         <v>1989</v>
       </c>
       <c r="H500">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="I500" s="2" t="s">
         <v>16</v>
@@ -21196,7 +21196,7 @@
         <v>1993</v>
       </c>
       <c r="H501">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="I501" s="2" t="s">
         <v>16</v>
@@ -21225,7 +21225,7 @@
         <v>1997</v>
       </c>
       <c r="H502">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="I502" s="2" t="s">
         <v>16</v>
@@ -21254,7 +21254,7 @@
         <v>2001</v>
       </c>
       <c r="H503">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="I503" s="2" t="s">
         <v>16</v>
@@ -21283,7 +21283,7 @@
         <v>2005</v>
       </c>
       <c r="H504">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I504" s="2" t="s">
         <v>16</v>
@@ -21312,7 +21312,7 @@
         <v>2009</v>
       </c>
       <c r="H505">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="I505" s="2" t="s">
         <v>16</v>
@@ -21341,7 +21341,7 @@
         <v>2013</v>
       </c>
       <c r="H506">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="I506" s="2" t="s">
         <v>16</v>
@@ -21370,7 +21370,7 @@
         <v>2017</v>
       </c>
       <c r="H507">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I507" s="2" t="s">
         <v>16</v>
@@ -21399,7 +21399,7 @@
         <v>2021</v>
       </c>
       <c r="H508">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="I508" s="2" t="s">
         <v>16</v>
@@ -21428,7 +21428,7 @@
         <v>2025</v>
       </c>
       <c r="H509">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="I509" s="2" t="s">
         <v>16</v>
@@ -21457,7 +21457,7 @@
         <v>2029</v>
       </c>
       <c r="H510">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="I510" s="2" t="s">
         <v>16</v>
@@ -21486,7 +21486,7 @@
         <v>2033</v>
       </c>
       <c r="H511">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="I511" s="2" t="s">
         <v>16</v>
@@ -21515,7 +21515,7 @@
         <v>2037</v>
       </c>
       <c r="H512">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I512" s="2" t="s">
         <v>16</v>
@@ -21544,7 +21544,7 @@
         <v>2041</v>
       </c>
       <c r="H513">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I513" s="2" t="s">
         <v>16</v>
@@ -21573,7 +21573,7 @@
         <v>2045</v>
       </c>
       <c r="H514">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="I514" s="2" t="s">
         <v>16</v>
@@ -21602,7 +21602,7 @@
         <v>2049</v>
       </c>
       <c r="H515">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="I515" s="2" t="s">
         <v>16</v>
@@ -21631,7 +21631,7 @@
         <v>2053</v>
       </c>
       <c r="H516">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="I516" s="2" t="s">
         <v>16</v>
@@ -21660,7 +21660,7 @@
         <v>2057</v>
       </c>
       <c r="H517">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="I517" s="2" t="s">
         <v>16</v>
@@ -21689,7 +21689,7 @@
         <v>2061</v>
       </c>
       <c r="H518">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="I518" s="2" t="s">
         <v>16</v>
@@ -21718,7 +21718,7 @@
         <v>2065</v>
       </c>
       <c r="H519">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="I519" s="2" t="s">
         <v>16</v>
@@ -21747,7 +21747,7 @@
         <v>2069</v>
       </c>
       <c r="H520">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="I520" s="2" t="s">
         <v>16</v>
@@ -21776,7 +21776,7 @@
         <v>2073</v>
       </c>
       <c r="H521">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I521" s="2" t="s">
         <v>16</v>
@@ -29144,7 +29144,7 @@
         <v>2077</v>
       </c>
       <c r="B4">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -29152,7 +29152,7 @@
         <v>2078</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>